<commit_message>
close out the numeric decisions
Mount of Slaanesh keeps Leadership 8; the wiki's 9 is the error, not the
catalogue.

Ghal Maraz at 180 is deliberate. Karl Franz must take exactly one of Ghal
Maraz at 180 or the Reikland Runefang at 100, and the Weapon group already
enforces that with min 1 and max 1 - so the wiki's 0 just reflects the item
not being separately priced there. Checked the constraints rather than
taking it on trust; they are right.

Every points and statline row is now settled. 64 rows remain, all of them
rules text: 57 with no wiki coverage and 7 ambiguous, 5 of which are the
long rules held back for summarising.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/judgement-calls.xlsx
+++ b/docs/judgement-calls.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Decisions" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Decisions'!$A$2:$J$69</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Decisions'!$A$2:$J$67</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -689,7 +689,7 @@
         </is>
       </c>
       <c r="B29" s="4">
-        <f>COUNTBLANK(Decisions!$I$4:$I$69)</f>
+        <f>COUNTBLANK(Decisions!$I$4:$I$67)</f>
         <v/>
       </c>
     </row>
@@ -704,7 +704,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J69"/>
+  <dimension ref="A1:J67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -3030,7 +3030,7 @@
       </c>
       <c r="B54" s="8" t="inlineStr">
         <is>
-          <t>Warlock Engineer</t>
+          <t>Warlock Master</t>
         </is>
       </c>
       <c r="C54" s="9" t="inlineStr">
@@ -3055,12 +3055,12 @@
       </c>
       <c r="G54" s="9" t="inlineStr">
         <is>
-          <t>/unit/warlock-engineer (1.00)</t>
+          <t>/unit/master (0.80)</t>
         </is>
       </c>
       <c r="H54" s="10" t="inlineStr">
         <is>
-          <t>https://6th.whfb.app/unit/warlock-engineer</t>
+          <t>https://6th.whfb.app/unit/master</t>
         </is>
       </c>
       <c r="I54" s="11" t="n"/>
@@ -3630,101 +3630,13 @@
       <c r="I67" s="11" t="n"/>
       <c r="J67" s="11" t="n"/>
     </row>
-    <row r="68">
-      <c r="A68" s="8" t="inlineStr">
-        <is>
-          <t>Points cost</t>
-        </is>
-      </c>
-      <c r="B68" s="8" t="inlineStr">
-        <is>
-          <t>Ghal Maraz</t>
-        </is>
-      </c>
-      <c r="C68" s="9" t="inlineStr">
-        <is>
-          <t>Emperor Karl Franz &gt; Weapon</t>
-        </is>
-      </c>
-      <c r="D68" s="8" t="inlineStr">
-        <is>
-          <t>The Empire.cat</t>
-        </is>
-      </c>
-      <c r="E68" s="9" t="inlineStr">
-        <is>
-          <t>catalogue and wiki disagree on cost</t>
-        </is>
-      </c>
-      <c r="F68" s="9" t="inlineStr">
-        <is>
-          <t>catalogue: 180</t>
-        </is>
-      </c>
-      <c r="G68" s="9" t="inlineStr">
-        <is>
-          <t>wiki: 0</t>
-        </is>
-      </c>
-      <c r="H68" s="10" t="inlineStr">
-        <is>
-          <t>https://6th.whfb.app/magic-item/ghal-maraz</t>
-        </is>
-      </c>
-      <c r="I68" s="11" t="n"/>
-      <c r="J68" s="11" t="n"/>
-    </row>
-    <row r="69">
-      <c r="A69" s="8" t="inlineStr">
-        <is>
-          <t>Unit statline</t>
-        </is>
-      </c>
-      <c r="B69" s="8" t="inlineStr">
-        <is>
-          <t>Mount of Slaanesh</t>
-        </is>
-      </c>
-      <c r="C69" s="9" t="inlineStr">
-        <is>
-          <t>Mounted Daemonettes &gt; Mounted Daemonettes</t>
-        </is>
-      </c>
-      <c r="D69" s="8" t="inlineStr">
-        <is>
-          <t>Forces of Chaos.cat</t>
-        </is>
-      </c>
-      <c r="E69" s="9" t="inlineStr">
-        <is>
-          <t>1 characteristic(s) differ</t>
-        </is>
-      </c>
-      <c r="F69" s="9" t="inlineStr">
-        <is>
-          <t>catalogue as is</t>
-        </is>
-      </c>
-      <c r="G69" s="9" t="inlineStr">
-        <is>
-          <t>wiki: Ld 8-&gt;9</t>
-        </is>
-      </c>
-      <c r="H69" s="10" t="inlineStr">
-        <is>
-          <t>https://6th.whfb.app/unit/mount-of-slaanesh</t>
-        </is>
-      </c>
-      <c r="I69" s="11" t="n"/>
-      <c r="J69" s="11" t="n"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A2:J69"/>
+  <autoFilter ref="A2:J67"/>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="I4:I69" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I4:I67" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Option A,Option B,Leave as is,Rename catalogue,Needs more thought"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3780,8 +3692,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H64" r:id="rId49"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H65" r:id="rId50"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H66" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H68" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H69" r:id="rId53"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>